<commit_message>
Add STA 220 Files
</commit_message>
<xml_diff>
--- a/statistics/spreadsheet_videos.xlsx
+++ b/statistics/spreadsheet_videos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\omega\Documents\GitHub\prof-sears.github.io\statistics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAFE2914-18BB-4B9D-9556-A3EF8D74A012}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9388053B-CE2A-40E5-9E08-8BE469CC4FC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{ADFFA339-263D-47E5-A4A3-FCE92E063BAC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ADFFA339-263D-47E5-A4A3-FCE92E063BAC}"/>
   </bookViews>
   <sheets>
     <sheet name="Introduction" sheetId="1" r:id="rId1"/>
@@ -2143,7 +2143,7 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -2151,15 +2151,18 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="3"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="8"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="7" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="2" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="3"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="6"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="8"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="5" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2171,10 +2174,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="5" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="7" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -2533,76 +2532,76 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
     </row>
     <row r="2" spans="1:13" ht="18.75" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="4"/>
+      <c r="B2" s="8"/>
       <c r="G2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9"/>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-      <c r="M2" s="9"/>
+      <c r="I2" s="10"/>
+      <c r="J2" s="10"/>
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3">
         <v>1</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="5">
-        <f>COUNT(A3:B16)</f>
+      <c r="E3" s="3">
+        <f>COUNT(A3:B17)</f>
         <v>10</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="11"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
+      <c r="I3" s="12"/>
+      <c r="J3" s="12"/>
+      <c r="K3" s="12"/>
+      <c r="L3" s="12"/>
+      <c r="M3" s="12"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4">
         <v>2</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="3">
         <f>COUNTA(A3:B17)</f>
         <v>20</v>
       </c>
@@ -2611,7 +2610,7 @@
       <c r="A5" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="12">
+      <c r="B5">
         <v>3</v>
       </c>
     </row>
@@ -2619,7 +2618,7 @@
       <c r="A6" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6">
         <v>4</v>
       </c>
     </row>
@@ -2627,7 +2626,7 @@
       <c r="A7" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7">
         <v>5</v>
       </c>
     </row>
@@ -2635,7 +2634,7 @@
       <c r="A8" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8">
         <v>6</v>
       </c>
     </row>
@@ -2643,7 +2642,7 @@
       <c r="A9" t="s">
         <v>0</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9">
         <v>7</v>
       </c>
     </row>
@@ -2651,7 +2650,7 @@
       <c r="A10" t="s">
         <v>1</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10">
         <v>8</v>
       </c>
     </row>
@@ -2659,7 +2658,7 @@
       <c r="A11" t="s">
         <v>2</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11">
         <v>9</v>
       </c>
     </row>
@@ -2667,7 +2666,7 @@
       <c r="A12" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12">
         <v>10</v>
       </c>
     </row>
@@ -2713,11 +2712,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:30" x14ac:dyDescent="0.25">
-      <c r="AB1" s="13" t="s">
+      <c r="AB1" s="6" t="s">
         <v>636</v>
       </c>
-      <c r="AC1" s="13"/>
-      <c r="AD1" s="5">
+      <c r="AC1" s="6"/>
+      <c r="AD1" s="3">
         <f>COUNTA(B4:B2000)</f>
         <v>572</v>
       </c>

</xml_diff>